<commit_message>
fix: update game states data in CSV for improved accuracy
</commit_message>
<xml_diff>
--- a/csv/game states.xlsx
+++ b/csv/game states.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e8b29edc4376667/Projects/Python/at_bat/csv/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Python\at_bat\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="421" documentId="8_{1E7C1C6B-8C31-4479-B74A-66C136A4727D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A0C74FE-86B6-4C81-A24D-E797EDC25FC0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD31C8F7-EFDF-4F41-8B96-52DB47513BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F5CA1E43-766A-4086-8122-BB1D980A4810}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5CA1E43-766A-4086-8122-BB1D980A4810}"/>
   </bookViews>
   <sheets>
     <sheet name="nonsortable" sheetId="2" r:id="rId1"/>
@@ -538,10 +538,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -842,16 +838,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B849384-B473-4938-862B-0224328C5BC9}">
   <dimension ref="A1:F61"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" style="1"/>
-    <col min="4" max="4" width="33.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.1796875" style="2"/>
+    <col min="1" max="1" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="33.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -871,7 +867,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
@@ -888,7 +884,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6" t="s">
@@ -904,7 +900,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -915,7 +911,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -926,7 +922,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -940,7 +936,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -951,7 +947,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -962,7 +958,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>6</v>
       </c>
@@ -980,7 +976,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6" t="s">
@@ -993,7 +989,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1004,7 +1000,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1018,7 +1014,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
@@ -1031,7 +1027,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1045,7 +1041,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1056,7 +1052,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1067,7 +1063,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1078,7 +1074,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1089,7 +1085,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1100,7 +1096,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1111,7 +1107,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1122,7 +1118,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1133,7 +1129,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1144,7 +1140,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1155,7 +1151,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1166,7 +1162,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1177,7 +1173,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1188,7 +1184,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1199,7 +1195,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -1210,7 +1206,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1221,7 +1217,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1232,7 +1228,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -1243,7 +1239,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -1257,7 +1253,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -1268,7 +1264,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6" t="s">
@@ -1281,7 +1277,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -1292,7 +1288,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -1303,7 +1299,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
@@ -1314,7 +1310,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -1325,7 +1321,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -1336,7 +1332,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -1347,7 +1343,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -1358,7 +1354,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1369,7 +1365,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -1380,7 +1376,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="1" t="s">
@@ -1394,7 +1390,7 @@
       </c>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="1" t="s">
@@ -1406,7 +1402,7 @@
       </c>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>7</v>
       </c>
@@ -1426,7 +1422,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -1440,7 +1436,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="6"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1451,7 +1447,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -1465,7 +1461,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6" t="s">
@@ -1481,7 +1477,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -1492,7 +1488,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -1506,7 +1502,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -1517,7 +1513,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -1531,7 +1527,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6" t="s">
@@ -1544,7 +1540,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -1555,7 +1551,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -1566,7 +1562,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6" t="s">
@@ -1582,7 +1578,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -1594,7 +1590,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
       <c r="D61" s="5"/>

</xml_diff>